<commit_message>
fix: layout box for excel in issue sheet
</commit_message>
<xml_diff>
--- a/src/lib/Site Activities.xlsx
+++ b/src/lib/Site Activities.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A648F86-59D1-4F98-B43F-672E7417ABE1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C88B3A91-955F-4996-A65F-437C1BDCE2D6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12120" yWindow="1800" windowWidth="13860" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3810" yWindow="2370" windowWidth="14880" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="7. Site Photos" sheetId="11" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="11">
   <si>
     <t/>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t xml:space="preserve">Action by: </t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -254,29 +257,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -285,59 +270,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -696,303 +702,335 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
     </row>
     <row r="5" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
     </row>
     <row r="6" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
     </row>
     <row r="7" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="11"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="13"/>
-      <c r="G7" s="7"/>
+      <c r="B7" s="5"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="7"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="10"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="8"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="3"/>
     </row>
     <row r="9" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="12"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="15"/>
-      <c r="G9" s="7"/>
+      <c r="B9" s="6"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="9"/>
+      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="B10" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
     </row>
     <row r="11" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="11"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="13"/>
-      <c r="G11" s="7"/>
+      <c r="B11" s="5"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="7"/>
+      <c r="G11" s="2"/>
     </row>
     <row r="12" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="10"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="8"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="3"/>
     </row>
     <row r="13" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="12"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="15"/>
-      <c r="G13" s="7"/>
+      <c r="B13" s="6"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="9"/>
+      <c r="G13" s="2"/>
     </row>
     <row r="14" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="B14" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
     </row>
     <row r="15" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="11"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="13"/>
-      <c r="G15" s="7"/>
+      <c r="B15" s="5"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="7"/>
+      <c r="G15" s="2"/>
     </row>
     <row r="16" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="10"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="8"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="3"/>
     </row>
     <row r="17" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="12"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="15"/>
-      <c r="G17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="9"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="B18" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
     </row>
     <row r="19" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="11"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="13"/>
-      <c r="G19" s="7"/>
+      <c r="B19" s="5"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="7"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="10"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="8"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="3"/>
     </row>
     <row r="21" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="12"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="15"/>
-      <c r="G21" s="7"/>
+      <c r="B21" s="6"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="9"/>
+      <c r="G21" s="2"/>
     </row>
     <row r="22" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="B22" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
     </row>
     <row r="23" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
     </row>
     <row r="24" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="11"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="13"/>
-      <c r="G24" s="7"/>
+      <c r="B24" s="5"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="7"/>
+      <c r="G24" s="2"/>
     </row>
     <row r="25" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="10"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="8"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="3"/>
     </row>
     <row r="26" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="12"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="15"/>
-      <c r="G26" s="7"/>
+      <c r="B26" s="6"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="9"/>
+      <c r="G26" s="2"/>
     </row>
     <row r="27" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="B27" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
     </row>
     <row r="28" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="11"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="13"/>
-      <c r="G28" s="7"/>
+      <c r="B28" s="5"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="7"/>
+      <c r="G28" s="2"/>
     </row>
     <row r="29" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="10"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="8"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="3"/>
     </row>
     <row r="30" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="12"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="15"/>
-      <c r="G30" s="7"/>
+      <c r="B30" s="6"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="9"/>
+      <c r="G30" s="2"/>
     </row>
     <row r="31" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
+      <c r="B31" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
     </row>
     <row r="32" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="11"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="13"/>
-      <c r="G32" s="7"/>
+      <c r="B32" s="5"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="7"/>
+      <c r="G32" s="2"/>
     </row>
     <row r="33" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="10"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="8"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="3"/>
     </row>
     <row r="34" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="12"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="15"/>
-      <c r="G34" s="7"/>
+      <c r="B34" s="6"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="9"/>
+      <c r="G34" s="2"/>
     </row>
     <row r="35" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
+      <c r="B35" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C35" s="14"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
     </row>
     <row r="36" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="11"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="13"/>
-      <c r="G36" s="7"/>
+      <c r="B36" s="5"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="7"/>
+      <c r="G36" s="2"/>
     </row>
     <row r="37" spans="2:7" ht="170.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="10"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="8"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="3"/>
     </row>
     <row r="38" spans="2:7" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="12"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="15"/>
-      <c r="G38" s="7"/>
+      <c r="B38" s="6"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="9"/>
+      <c r="G38" s="2"/>
     </row>
     <row r="39" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+      <c r="B39" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="B23:G23"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="B27:D27"/>
@@ -1001,18 +1039,6 @@
     <mergeCell ref="E31:G31"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="E35:G35"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B6:G6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -1032,407 +1058,433 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="4" spans="2:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
     </row>
     <row r="5" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="33">
+      <c r="B5" s="21">
         <v>1</v>
       </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
     </row>
     <row r="6" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="31"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="32"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="31"/>
     </row>
     <row r="9" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="32"/>
+      <c r="B9" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="28"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="31"/>
     </row>
     <row r="10" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="5"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="32"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="31"/>
     </row>
     <row r="11" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="32"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="31"/>
     </row>
     <row r="12" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="5"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="32"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="31"/>
     </row>
     <row r="13" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="5"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="32"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="31"/>
     </row>
     <row r="14" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="5"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="32"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="31"/>
     </row>
     <row r="15" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="5"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="32"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="31"/>
     </row>
     <row r="16" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="5"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="32"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="31"/>
     </row>
     <row r="17" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="32"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="31"/>
     </row>
     <row r="18" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="3"/>
+      <c r="B18" s="35"/>
       <c r="C18" s="29"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="23"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="32"/>
     </row>
     <row r="19" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="33">
+      <c r="B19" s="21">
         <v>2</v>
       </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
     </row>
     <row r="20" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="22"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="23"/>
     </row>
     <row r="21" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="31"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="30"/>
     </row>
     <row r="22" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="30"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="32"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="31"/>
     </row>
     <row r="23" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" s="25"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="32"/>
+      <c r="B23" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="31"/>
     </row>
     <row r="24" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="5"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="32"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="31"/>
     </row>
     <row r="25" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="5"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="32"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="31"/>
     </row>
     <row r="26" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="5"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="32"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="31"/>
     </row>
     <row r="27" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="5"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="32"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="31"/>
     </row>
     <row r="28" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="5"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="32"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="31"/>
     </row>
     <row r="29" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="5"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="32"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="31"/>
     </row>
     <row r="30" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="5"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="32"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="31"/>
     </row>
     <row r="31" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="25"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="32"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="31"/>
     </row>
     <row r="32" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="3"/>
+      <c r="B32" s="35"/>
       <c r="C32" s="29"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="23"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="32"/>
     </row>
     <row r="33" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="33">
+      <c r="B33" s="21">
         <v>3</v>
       </c>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
     </row>
     <row r="34" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D34" s="4"/>
-      <c r="E34" s="22"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="23"/>
     </row>
     <row r="35" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="35" t="s">
+      <c r="B35" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C35" s="24"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="31"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="30"/>
     </row>
     <row r="36" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="30"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="32"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="31"/>
     </row>
     <row r="37" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="32"/>
+      <c r="B37" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" s="28"/>
+      <c r="D37" s="33"/>
+      <c r="E37" s="31"/>
     </row>
     <row r="38" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="5"/>
-      <c r="C38" s="25"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="32"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="31"/>
     </row>
     <row r="39" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="5"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="32"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="31"/>
     </row>
     <row r="40" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="5"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="32"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="31"/>
     </row>
     <row r="41" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="5"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="32"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="31"/>
     </row>
     <row r="42" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="5"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="32"/>
+      <c r="B42" s="34"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="31"/>
     </row>
     <row r="43" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="5"/>
-      <c r="C43" s="25"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="32"/>
+      <c r="B43" s="34"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="31"/>
     </row>
     <row r="44" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="5"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="32"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="45" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C45" s="25"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="32"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="3"/>
+      <c r="B46" s="35"/>
       <c r="C46" s="29"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="23"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="32"/>
     </row>
     <row r="47" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="33">
+      <c r="B47" s="21">
         <v>4</v>
       </c>
-      <c r="C47" s="34"/>
-      <c r="D47" s="34"/>
-      <c r="E47" s="34"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
     </row>
     <row r="48" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="27" t="s">
+      <c r="B48" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C48" s="22" t="s">
+      <c r="C48" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D48" s="4"/>
-      <c r="E48" s="22"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="23"/>
     </row>
     <row r="49" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="35" t="s">
+      <c r="B49" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C49" s="24"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="31"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="30"/>
     </row>
     <row r="50" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="30"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="32"/>
+      <c r="B50" s="26"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="31"/>
     </row>
     <row r="51" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C51" s="25"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="32"/>
+      <c r="B51" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="C51" s="28"/>
+      <c r="D51" s="33"/>
+      <c r="E51" s="31"/>
     </row>
     <row r="52" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="5"/>
-      <c r="C52" s="25"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="32"/>
+      <c r="B52" s="34"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="33"/>
+      <c r="E52" s="31"/>
     </row>
     <row r="53" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="5"/>
-      <c r="C53" s="25"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="32"/>
+      <c r="B53" s="34"/>
+      <c r="C53" s="28"/>
+      <c r="D53" s="33"/>
+      <c r="E53" s="31"/>
     </row>
     <row r="54" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="5"/>
-      <c r="C54" s="25"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="32"/>
+      <c r="B54" s="34"/>
+      <c r="C54" s="28"/>
+      <c r="D54" s="33"/>
+      <c r="E54" s="31"/>
     </row>
     <row r="55" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="5"/>
-      <c r="C55" s="25"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="32"/>
+      <c r="B55" s="34"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="33"/>
+      <c r="E55" s="31"/>
     </row>
     <row r="56" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="5"/>
-      <c r="C56" s="25"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="32"/>
+      <c r="B56" s="34"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="31"/>
     </row>
     <row r="57" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="5"/>
-      <c r="C57" s="25"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="32"/>
+      <c r="B57" s="34"/>
+      <c r="C57" s="28"/>
+      <c r="D57" s="33"/>
+      <c r="E57" s="31"/>
     </row>
     <row r="58" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="5"/>
-      <c r="C58" s="25"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="32"/>
+      <c r="B58" s="34"/>
+      <c r="C58" s="28"/>
+      <c r="D58" s="33"/>
+      <c r="E58" s="31"/>
     </row>
     <row r="59" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C59" s="25"/>
-      <c r="D59" s="26"/>
-      <c r="E59" s="32"/>
+      <c r="C59" s="28"/>
+      <c r="D59" s="33"/>
+      <c r="E59" s="31"/>
     </row>
     <row r="60" spans="2:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="3"/>
+      <c r="B60" s="35"/>
       <c r="C60" s="29"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="23"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="E7:E18"/>
+    <mergeCell ref="C7:C18"/>
+    <mergeCell ref="B9:B16"/>
+    <mergeCell ref="D8:D17"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C32"/>
+    <mergeCell ref="E21:E32"/>
+    <mergeCell ref="D22:D31"/>
+    <mergeCell ref="B23:B30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C46"/>
+    <mergeCell ref="E35:E46"/>
+    <mergeCell ref="D36:D45"/>
+    <mergeCell ref="B37:B44"/>
+    <mergeCell ref="B45:B46"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="C48:E48"/>
     <mergeCell ref="B49:B50"/>
@@ -1441,32 +1493,6 @@
     <mergeCell ref="D50:D59"/>
     <mergeCell ref="B51:B58"/>
     <mergeCell ref="B59:B60"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C46"/>
-    <mergeCell ref="E35:E46"/>
-    <mergeCell ref="D36:D45"/>
-    <mergeCell ref="B37:B44"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C32"/>
-    <mergeCell ref="E21:E32"/>
-    <mergeCell ref="D22:D31"/>
-    <mergeCell ref="B23:B30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="E7:E18"/>
-    <mergeCell ref="C7:C18"/>
-    <mergeCell ref="B9:B16"/>
-    <mergeCell ref="D8:D17"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>